<commit_message>
Add Brand and Type/Model to PPT data Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ReNvkBKePFXKJiXPJLaYQp
</commit_message>
<xml_diff>
--- a/PPT_Freight_Insurance_FOB.xlsx
+++ b/PPT_Freight_Insurance_FOB.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPT Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PPT Data'!$A$1:$I$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PPT Data'!$A$1:$K$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:K185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -438,6 +438,8 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,6 +488,16 @@
           <t>Currency</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Type/Model</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -523,6 +535,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,6 +582,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -597,6 +629,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -634,6 +676,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -671,6 +723,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -708,6 +770,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -745,6 +817,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -782,6 +864,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -819,6 +911,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -856,6 +958,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -893,6 +1005,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -930,6 +1052,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -967,6 +1099,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1004,6 +1146,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1041,6 +1193,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1078,6 +1240,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1115,6 +1287,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1152,6 +1334,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1189,6 +1381,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1226,6 +1428,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1263,6 +1475,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1300,6 +1522,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>930E-5</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1337,6 +1569,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1374,6 +1616,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>930E-5</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1411,6 +1663,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>830E-1</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1448,6 +1710,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1485,6 +1757,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>930E-4</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1522,6 +1804,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1559,6 +1851,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>930E-4</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1596,6 +1898,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1633,6 +1945,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1670,6 +1992,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1707,6 +2039,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1744,6 +2086,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1781,6 +2133,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1818,6 +2180,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1855,6 +2227,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1892,6 +2274,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1929,6 +2321,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1966,6 +2368,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2003,6 +2415,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>930E-5</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2040,6 +2462,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>930E-5</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2077,6 +2509,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2114,6 +2556,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>930E-5</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2151,6 +2603,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2188,6 +2650,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2225,6 +2697,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2262,6 +2744,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>930E-4</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2299,6 +2791,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2336,6 +2838,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>930E-4</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2373,6 +2885,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2410,6 +2932,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2447,6 +2979,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2484,6 +3026,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2521,6 +3073,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2558,6 +3120,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2595,6 +3167,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2632,6 +3214,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2669,6 +3261,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Hitachi</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>EH4000AC-3</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2706,6 +3308,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2743,6 +3355,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2780,6 +3402,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2817,6 +3449,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2854,6 +3496,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2891,6 +3543,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2928,6 +3590,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2965,6 +3637,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3002,6 +3684,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3039,6 +3731,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3076,6 +3778,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3113,6 +3825,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3150,6 +3872,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>830-5</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3187,6 +3919,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Epiroc</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>MT65</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3224,6 +3966,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3261,6 +4013,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3298,6 +4060,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>NHL</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>NTE-360</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3335,6 +4107,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3372,6 +4154,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3409,6 +4201,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3446,6 +4248,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>930E-4</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3483,6 +4295,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3520,6 +4342,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3557,6 +4389,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Hitachi</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>EH4000AC-3</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3594,6 +4436,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3631,6 +4483,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3668,6 +4530,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3705,6 +4577,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3742,6 +4624,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3779,6 +4671,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3816,6 +4718,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3853,6 +4765,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3890,6 +4812,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3927,6 +4859,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3964,6 +4906,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4001,6 +4953,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4038,6 +5000,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>793F</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4075,6 +5047,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>793F</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4112,6 +5094,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>930E</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4149,6 +5141,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>793E</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4186,6 +5188,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>795F</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4223,6 +5235,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4260,6 +5282,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4297,6 +5329,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4334,6 +5376,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4371,6 +5423,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4408,6 +5470,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4445,6 +5517,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4482,6 +5564,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4519,6 +5611,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4556,6 +5658,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>830E-AC</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4593,6 +5705,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>HD830-5</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4630,6 +5752,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4667,6 +5799,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>830E-5</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4704,6 +5846,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4741,6 +5893,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4778,6 +5940,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>930-5</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4815,6 +5987,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4852,6 +6034,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4889,6 +6081,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4926,6 +6128,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4963,6 +6175,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5000,6 +6222,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5037,6 +6269,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>830E</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5074,6 +6316,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5111,6 +6363,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Sandvik</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>TH663i</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5148,6 +6410,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5185,6 +6457,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5222,6 +6504,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>777F</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5259,6 +6551,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>789D</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5296,6 +6598,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5333,6 +6645,14 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>785</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5370,6 +6690,14 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>785</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5407,6 +6735,14 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K134" t="n">
+        <v>785</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5444,6 +6780,14 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K135" t="n">
+        <v>785</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5481,6 +6825,14 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>785</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5518,6 +6870,14 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K137" t="n">
+        <v>785</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5555,6 +6915,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>785NG</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5592,6 +6962,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>785NG</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5629,6 +7009,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5666,6 +7056,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5703,6 +7103,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5740,6 +7150,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5777,6 +7197,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5814,6 +7244,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5851,6 +7291,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5888,6 +7338,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5925,6 +7385,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5962,6 +7432,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5999,6 +7479,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6036,6 +7526,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6073,6 +7573,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6110,6 +7620,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6147,6 +7667,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6184,6 +7714,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6221,6 +7761,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6258,6 +7808,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6295,6 +7855,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6332,6 +7902,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6369,6 +7949,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6406,6 +7996,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6443,6 +8043,16 @@
           <t>AUD</t>
         </is>
       </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>785D</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6480,6 +8090,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>777E</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -6517,6 +8137,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>777E</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6554,6 +8184,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>777E</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6591,6 +8231,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>777E</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6628,6 +8278,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>777E</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -6665,6 +8325,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>777E</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6702,6 +8372,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -6739,6 +8419,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6776,6 +8466,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6813,6 +8513,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -6850,6 +8560,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6887,6 +8607,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -6924,6 +8654,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Hitachi</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>EH4000AC-3</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -6961,6 +8701,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Caterpillar</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>785C</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6998,6 +8748,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -7035,6 +8795,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -7072,6 +8842,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7109,6 +8889,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -7146,6 +8936,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7183,6 +8983,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -7220,6 +9030,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -7257,6 +9077,16 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>HD785-7</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -7294,9 +9124,19 @@
           <t>USD</t>
         </is>
       </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Komatsu</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>930E-4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I185"/>
+  <autoFilter ref="A1:K185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Derive Brand and Type/Model from goods description with normalized naming
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ReNvkBKePFXKJiXPJLaYQp
</commit_message>
<xml_diff>
--- a/PPT_Freight_Insurance_FOB.xlsx
+++ b/PPT_Freight_Insurance_FOB.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>930E</t>
+          <t>930E-4</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>930E</t>
+          <t>930E-4</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>830E-1</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -1900,12 +1900,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Caterpillar</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>777G</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3597,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3973,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>NTE-360</t>
+          <t>NTE360</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E-4SE</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -5237,12 +5237,12 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5284,12 +5284,12 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5331,12 +5331,12 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5378,12 +5378,12 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5425,12 +5425,12 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5519,12 +5519,12 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5566,12 +5566,12 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5613,12 +5613,12 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>830E</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5665,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>830E-AC</t>
+          <t>830E-1AC</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>HD830-5</t>
+          <t>830E-5</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>930-5</t>
+          <t>930E-5</t>
         </is>
       </c>
     </row>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785C/785D</t>
         </is>
       </c>
     </row>
@@ -6412,12 +6412,12 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>930E</t>
         </is>
       </c>
     </row>
@@ -6650,8 +6650,10 @@
           <t>Caterpillar</t>
         </is>
       </c>
-      <c r="K132" t="n">
-        <v>785</v>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>785</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -6695,8 +6697,10 @@
           <t>Caterpillar</t>
         </is>
       </c>
-      <c r="K133" t="n">
-        <v>785</v>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>785</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -6740,8 +6744,10 @@
           <t>Caterpillar</t>
         </is>
       </c>
-      <c r="K134" t="n">
-        <v>785</v>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>785</t>
+        </is>
       </c>
     </row>
     <row r="135">
@@ -6785,8 +6791,10 @@
           <t>Caterpillar</t>
         </is>
       </c>
-      <c r="K135" t="n">
-        <v>785</v>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>785</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -6830,8 +6838,10 @@
           <t>Caterpillar</t>
         </is>
       </c>
-      <c r="K136" t="n">
-        <v>785</v>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>785</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -6875,8 +6885,10 @@
           <t>Caterpillar</t>
         </is>
       </c>
-      <c r="K137" t="n">
-        <v>785</v>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>785</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -6922,7 +6934,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>785NG</t>
+          <t>785 Next Gen</t>
         </is>
       </c>
     </row>
@@ -6969,7 +6981,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>785NG</t>
+          <t>785 Next Gen</t>
         </is>
       </c>
     </row>
@@ -7340,12 +7352,12 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>HD785-7</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7451,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7498,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8297,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>777E</t>
+          <t>777D/777E</t>
         </is>
       </c>
     </row>
@@ -8515,12 +8527,12 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Hitachi</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>EH4000AC-3</t>
         </is>
       </c>
     </row>
@@ -8750,12 +8762,12 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Komatsu</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>HD785-7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge 785/777 variants, standardize buyer names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ReNvkBKePFXKJiXPJLaYQp
</commit_message>
<xml_diff>
--- a/PPT_Freight_Insurance_FOB.xlsx
+++ b/PPT_Freight_Insurance_FOB.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -554,7 +554,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -601,7 +601,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -648,7 +648,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -695,7 +695,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -742,7 +742,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -836,7 +836,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -977,7 +977,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ANGLO AMERICA</t>
+          <t>Anglo American</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ANGLO COAL CAPCC</t>
+          <t>Anglo Coal Capcoal Management</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ANGLO COAL CAPCC</t>
+          <t>Anglo Coal Capcoal Management</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINNERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MRL ASSET MANAGE</t>
+          <t>MRL Asset Management Pty Limited</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -5019,7 +5019,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PILBARA IRON COMP</t>
+          <t>Pilbara Iron Company Services</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -5724,7 +5724,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>MRL ASSET MANAGE</t>
+          <t>MRL Asset Management Pty Limited</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -6194,7 +6194,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>HAMERSLEY IRON PT</t>
+          <t>Hamersley Iron Pty Limited</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>785C/785D</t>
+          <t>785</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -6523,7 +6523,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>AUSTIN ENGINEERIN</t>
+          <t>Austin Engineering Limited</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>QUAD EFFICIENT ENC</t>
+          <t>Quad Efficient Engineering Pty Limited</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>QUAD EFFICIENT ENC</t>
+          <t>Quad Efficient Engineering Pty Limited</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -6899,7 +6899,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>785 Next Gen</t>
+          <t>785</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>785 Next Gen</t>
+          <t>785</t>
         </is>
       </c>
     </row>
@@ -6993,7 +6993,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>MOROBE CONSOLIDA</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>MOROBE CONSOLIDA</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -7087,7 +7087,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>MOROBE CONSOLIDA</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>MOROBE CONSOLIDA</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>MOROBE CONSOLIDA</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -7228,7 +7228,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>MONROBE CONSOLII</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>MONROBE CONSOLII</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>MONROBE CONSOLII</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>MONROBE CONSOLII</t>
+          <t>Morobe Consolidated Goldfields Limited</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -7416,7 +7416,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>DURATRAY INTERNAT</t>
+          <t>Duratray International Pty Ltd</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -7510,7 +7510,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -7792,7 +7792,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -7933,7 +7933,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -7980,7 +7980,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>LIHIR GOLD LIMITED</t>
+          <t>Lihir Gold Limited</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>KIBALI GOLD MINES</t>
+          <t>Kibali Gold Mines SA KGM</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>KIBALI GOLD MINES</t>
+          <t>Kibali Gold Mines SA KGM</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -8168,7 +8168,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>KIBALI GOLD MINES</t>
+          <t>Kibali Gold Mines SA KGM</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -8215,7 +8215,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>KIBALI GOLD MINES</t>
+          <t>Kibali Gold Mines SA KGM</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>GOUNKOTO SA</t>
+          <t>Gounkoto SA</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -8297,7 +8297,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>777D/777E</t>
+          <t>777</t>
         </is>
       </c>
     </row>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>FEKOLA SA</t>
+          <t>Fekola SA</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>GOUNKOTO</t>
+          <t>Gounkoto SA</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>GOUNKOTO</t>
+          <t>Gounkoto SA</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>GOUNKOTO</t>
+          <t>Gounkoto SA</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>TATA STEEL LIMITED</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>THRIVENI SAINIK MIN</t>
+          <t>Thriveni Sainik Mining Private Limited</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>THRIVENI EARTHMOV</t>
+          <t>Thriveni Earthmovers and Infra Private</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>TATA STEEL LIMITED</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>TATA STEEL LIMITED</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>TATA STEEL LIMITED</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>TATA STEEL LIMITED</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>TATA STEEL LIMITED</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -9108,7 +9108,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>NEWMONT MEXICO</t>
+          <t>Newmont Mexico Minera Penasquito</t>
         </is>
       </c>
       <c r="C185" t="n">

</xml_diff>

<commit_message>
Add Insurance/Freight/FOB IDR columns and dark header style
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ReNvkBKePFXKJiXPJLaYQp
</commit_message>
<xml_diff>
--- a/PPT_Freight_Insurance_FOB.xlsx
+++ b/PPT_Freight_Insurance_FOB.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPT Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PPT Data'!$A$1:$K$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PPT Data'!$A$1:$N$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +32,15 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +50,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D3D3D"/>
+        <bgColor rgb="FF333300"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,10 +71,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K185"/>
+  <dimension ref="A1:N185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -440,62 +466,80 @@
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Goods Description</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Buyer Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Freight</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>FOB Value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Net Weight</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Type/Model</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Insurance IDR</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Freight IDR</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>FOB IDR</t>
         </is>
       </c>
     </row>
@@ -545,6 +589,18 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L2" s="4">
+        <f>$D2*IF($I2="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M2" s="4">
+        <f>$E2*IF($I2="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N2" s="4">
+        <f>$F2*IF($I2="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -592,6 +648,18 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L3" s="4">
+        <f>$D3*IF($I3="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M3" s="4">
+        <f>$E3*IF($I3="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N3" s="4">
+        <f>$F3*IF($I3="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -639,6 +707,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L4" s="4">
+        <f>$D4*IF($I4="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M4" s="4">
+        <f>$E4*IF($I4="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N4" s="4">
+        <f>$F4*IF($I4="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -686,6 +766,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L5" s="4">
+        <f>$D5*IF($I5="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
+        <f>$E5*IF($I5="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N5" s="4">
+        <f>$F5*IF($I5="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -733,6 +825,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L6" s="4">
+        <f>$D6*IF($I6="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M6" s="4">
+        <f>$E6*IF($I6="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N6" s="4">
+        <f>$F6*IF($I6="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -780,6 +884,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L7" s="4">
+        <f>$D7*IF($I7="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M7" s="4">
+        <f>$E7*IF($I7="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N7" s="4">
+        <f>$F7*IF($I7="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -827,6 +943,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L8" s="4">
+        <f>$D8*IF($I8="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
+        <f>$E8*IF($I8="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>$F8*IF($I8="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -874,6 +1002,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L9" s="4">
+        <f>$D9*IF($I9="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M9" s="4">
+        <f>$E9*IF($I9="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N9" s="4">
+        <f>$F9*IF($I9="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -921,6 +1061,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L10" s="4">
+        <f>$D10*IF($I10="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M10" s="4">
+        <f>$E10*IF($I10="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N10" s="4">
+        <f>$F10*IF($I10="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -968,6 +1120,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L11" s="4">
+        <f>$D11*IF($I11="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M11" s="4">
+        <f>$E11*IF($I11="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N11" s="4">
+        <f>$F11*IF($I11="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1015,6 +1179,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L12" s="4">
+        <f>$D12*IF($I12="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M12" s="4">
+        <f>$E12*IF($I12="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N12" s="4">
+        <f>$F12*IF($I12="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1062,6 +1238,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L13" s="4">
+        <f>$D13*IF($I13="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M13" s="4">
+        <f>$E13*IF($I13="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N13" s="4">
+        <f>$F13*IF($I13="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1109,6 +1297,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L14" s="4">
+        <f>$D14*IF($I14="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M14" s="4">
+        <f>$E14*IF($I14="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N14" s="4">
+        <f>$F14*IF($I14="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1156,6 +1356,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L15" s="4">
+        <f>$D15*IF($I15="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M15" s="4">
+        <f>$E15*IF($I15="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N15" s="4">
+        <f>$F15*IF($I15="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1203,6 +1415,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L16" s="4">
+        <f>$D16*IF($I16="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M16" s="4">
+        <f>$E16*IF($I16="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N16" s="4">
+        <f>$F16*IF($I16="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1250,6 +1474,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L17" s="4">
+        <f>$D17*IF($I17="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M17" s="4">
+        <f>$E17*IF($I17="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N17" s="4">
+        <f>$F17*IF($I17="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1297,6 +1533,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L18" s="4">
+        <f>$D18*IF($I18="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M18" s="4">
+        <f>$E18*IF($I18="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N18" s="4">
+        <f>$F18*IF($I18="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1344,6 +1592,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L19" s="4">
+        <f>$D19*IF($I19="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M19" s="4">
+        <f>$E19*IF($I19="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N19" s="4">
+        <f>$F19*IF($I19="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1391,6 +1651,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L20" s="4">
+        <f>$D20*IF($I20="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M20" s="4">
+        <f>$E20*IF($I20="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N20" s="4">
+        <f>$F20*IF($I20="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1438,6 +1710,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L21" s="4">
+        <f>$D21*IF($I21="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M21" s="4">
+        <f>$E21*IF($I21="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N21" s="4">
+        <f>$F21*IF($I21="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1485,6 +1769,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L22" s="4">
+        <f>$D22*IF($I22="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M22" s="4">
+        <f>$E22*IF($I22="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N22" s="4">
+        <f>$F22*IF($I22="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1532,6 +1828,18 @@
           <t>930E-5</t>
         </is>
       </c>
+      <c r="L23" s="4">
+        <f>$D23*IF($I23="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M23" s="4">
+        <f>$E23*IF($I23="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N23" s="4">
+        <f>$F23*IF($I23="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1579,6 +1887,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L24" s="4">
+        <f>$D24*IF($I24="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M24" s="4">
+        <f>$E24*IF($I24="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N24" s="4">
+        <f>$F24*IF($I24="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1626,6 +1946,18 @@
           <t>930E-5</t>
         </is>
       </c>
+      <c r="L25" s="4">
+        <f>$D25*IF($I25="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M25" s="4">
+        <f>$E25*IF($I25="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N25" s="4">
+        <f>$F25*IF($I25="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1673,6 +2005,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L26" s="4">
+        <f>$D26*IF($I26="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M26" s="4">
+        <f>$E26*IF($I26="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N26" s="4">
+        <f>$F26*IF($I26="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1720,6 +2064,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L27" s="4">
+        <f>$D27*IF($I27="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M27" s="4">
+        <f>$E27*IF($I27="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N27" s="4">
+        <f>$F27*IF($I27="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1767,6 +2123,18 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L28" s="4">
+        <f>$D28*IF($I28="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M28" s="4">
+        <f>$E28*IF($I28="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N28" s="4">
+        <f>$F28*IF($I28="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1814,6 +2182,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L29" s="4">
+        <f>$D29*IF($I29="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M29" s="4">
+        <f>$E29*IF($I29="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N29" s="4">
+        <f>$F29*IF($I29="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1861,6 +2241,18 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L30" s="4">
+        <f>$D30*IF($I30="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M30" s="4">
+        <f>$E30*IF($I30="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N30" s="4">
+        <f>$F30*IF($I30="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1908,6 +2300,18 @@
           <t>777G</t>
         </is>
       </c>
+      <c r="L31" s="4">
+        <f>$D31*IF($I31="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M31" s="4">
+        <f>$E31*IF($I31="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N31" s="4">
+        <f>$F31*IF($I31="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1955,6 +2359,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L32" s="4">
+        <f>$D32*IF($I32="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M32" s="4">
+        <f>$E32*IF($I32="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N32" s="4">
+        <f>$F32*IF($I32="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2002,6 +2418,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L33" s="4">
+        <f>$D33*IF($I33="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M33" s="4">
+        <f>$E33*IF($I33="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N33" s="4">
+        <f>$F33*IF($I33="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2049,6 +2477,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L34" s="4">
+        <f>$D34*IF($I34="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M34" s="4">
+        <f>$E34*IF($I34="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N34" s="4">
+        <f>$F34*IF($I34="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2096,6 +2536,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L35" s="4">
+        <f>$D35*IF($I35="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M35" s="4">
+        <f>$E35*IF($I35="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N35" s="4">
+        <f>$F35*IF($I35="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2143,6 +2595,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L36" s="4">
+        <f>$D36*IF($I36="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M36" s="4">
+        <f>$E36*IF($I36="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N36" s="4">
+        <f>$F36*IF($I36="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2190,6 +2654,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L37" s="4">
+        <f>$D37*IF($I37="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M37" s="4">
+        <f>$E37*IF($I37="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N37" s="4">
+        <f>$F37*IF($I37="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2237,6 +2713,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L38" s="4">
+        <f>$D38*IF($I38="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M38" s="4">
+        <f>$E38*IF($I38="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N38" s="4">
+        <f>$F38*IF($I38="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2284,6 +2772,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L39" s="4">
+        <f>$D39*IF($I39="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M39" s="4">
+        <f>$E39*IF($I39="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N39" s="4">
+        <f>$F39*IF($I39="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2331,6 +2831,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L40" s="4">
+        <f>$D40*IF($I40="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M40" s="4">
+        <f>$E40*IF($I40="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N40" s="4">
+        <f>$F40*IF($I40="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2378,6 +2890,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L41" s="4">
+        <f>$D41*IF($I41="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M41" s="4">
+        <f>$E41*IF($I41="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N41" s="4">
+        <f>$F41*IF($I41="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2425,6 +2949,18 @@
           <t>930E-5</t>
         </is>
       </c>
+      <c r="L42" s="4">
+        <f>$D42*IF($I42="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M42" s="4">
+        <f>$E42*IF($I42="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N42" s="4">
+        <f>$F42*IF($I42="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2472,6 +3008,18 @@
           <t>930E-5</t>
         </is>
       </c>
+      <c r="L43" s="4">
+        <f>$D43*IF($I43="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M43" s="4">
+        <f>$E43*IF($I43="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N43" s="4">
+        <f>$F43*IF($I43="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2519,6 +3067,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L44" s="4">
+        <f>$D44*IF($I44="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M44" s="4">
+        <f>$E44*IF($I44="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N44" s="4">
+        <f>$F44*IF($I44="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2566,6 +3126,18 @@
           <t>930E-5</t>
         </is>
       </c>
+      <c r="L45" s="4">
+        <f>$D45*IF($I45="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M45" s="4">
+        <f>$E45*IF($I45="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N45" s="4">
+        <f>$F45*IF($I45="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2613,6 +3185,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L46" s="4">
+        <f>$D46*IF($I46="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M46" s="4">
+        <f>$E46*IF($I46="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N46" s="4">
+        <f>$F46*IF($I46="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2660,6 +3244,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L47" s="4">
+        <f>$D47*IF($I47="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M47" s="4">
+        <f>$E47*IF($I47="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N47" s="4">
+        <f>$F47*IF($I47="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2707,6 +3303,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L48" s="4">
+        <f>$D48*IF($I48="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M48" s="4">
+        <f>$E48*IF($I48="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N48" s="4">
+        <f>$F48*IF($I48="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2754,6 +3362,18 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L49" s="4">
+        <f>$D49*IF($I49="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M49" s="4">
+        <f>$E49*IF($I49="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N49" s="4">
+        <f>$F49*IF($I49="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2801,6 +3421,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L50" s="4">
+        <f>$D50*IF($I50="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M50" s="4">
+        <f>$E50*IF($I50="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N50" s="4">
+        <f>$F50*IF($I50="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2848,6 +3480,18 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L51" s="4">
+        <f>$D51*IF($I51="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M51" s="4">
+        <f>$E51*IF($I51="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N51" s="4">
+        <f>$F51*IF($I51="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2895,6 +3539,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L52" s="4">
+        <f>$D52*IF($I52="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M52" s="4">
+        <f>$E52*IF($I52="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N52" s="4">
+        <f>$F52*IF($I52="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2942,6 +3598,18 @@
           <t>785C</t>
         </is>
       </c>
+      <c r="L53" s="4">
+        <f>$D53*IF($I53="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M53" s="4">
+        <f>$E53*IF($I53="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N53" s="4">
+        <f>$F53*IF($I53="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2989,6 +3657,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L54" s="4">
+        <f>$D54*IF($I54="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M54" s="4">
+        <f>$E54*IF($I54="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N54" s="4">
+        <f>$F54*IF($I54="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3036,6 +3716,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L55" s="4">
+        <f>$D55*IF($I55="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M55" s="4">
+        <f>$E55*IF($I55="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N55" s="4">
+        <f>$F55*IF($I55="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3083,6 +3775,18 @@
           <t>785C</t>
         </is>
       </c>
+      <c r="L56" s="4">
+        <f>$D56*IF($I56="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M56" s="4">
+        <f>$E56*IF($I56="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N56" s="4">
+        <f>$F56*IF($I56="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3130,6 +3834,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L57" s="4">
+        <f>$D57*IF($I57="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M57" s="4">
+        <f>$E57*IF($I57="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N57" s="4">
+        <f>$F57*IF($I57="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3177,6 +3893,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L58" s="4">
+        <f>$D58*IF($I58="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M58" s="4">
+        <f>$E58*IF($I58="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N58" s="4">
+        <f>$F58*IF($I58="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3224,6 +3952,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L59" s="4">
+        <f>$D59*IF($I59="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M59" s="4">
+        <f>$E59*IF($I59="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N59" s="4">
+        <f>$F59*IF($I59="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3271,6 +4011,18 @@
           <t>EH4000AC-3</t>
         </is>
       </c>
+      <c r="L60" s="4">
+        <f>$D60*IF($I60="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M60" s="4">
+        <f>$E60*IF($I60="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N60" s="4">
+        <f>$F60*IF($I60="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3318,6 +4070,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L61" s="4">
+        <f>$D61*IF($I61="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M61" s="4">
+        <f>$E61*IF($I61="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N61" s="4">
+        <f>$F61*IF($I61="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3365,6 +4129,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L62" s="4">
+        <f>$D62*IF($I62="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M62" s="4">
+        <f>$E62*IF($I62="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N62" s="4">
+        <f>$F62*IF($I62="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3412,6 +4188,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L63" s="4">
+        <f>$D63*IF($I63="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M63" s="4">
+        <f>$E63*IF($I63="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N63" s="4">
+        <f>$F63*IF($I63="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3459,6 +4247,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L64" s="4">
+        <f>$D64*IF($I64="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M64" s="4">
+        <f>$E64*IF($I64="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N64" s="4">
+        <f>$F64*IF($I64="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3506,6 +4306,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L65" s="4">
+        <f>$D65*IF($I65="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M65" s="4">
+        <f>$E65*IF($I65="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N65" s="4">
+        <f>$F65*IF($I65="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3553,6 +4365,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L66" s="4">
+        <f>$D66*IF($I66="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M66" s="4">
+        <f>$E66*IF($I66="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N66" s="4">
+        <f>$F66*IF($I66="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3600,6 +4424,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L67" s="4">
+        <f>$D67*IF($I67="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M67" s="4">
+        <f>$E67*IF($I67="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N67" s="4">
+        <f>$F67*IF($I67="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3647,6 +4483,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L68" s="4">
+        <f>$D68*IF($I68="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M68" s="4">
+        <f>$E68*IF($I68="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N68" s="4">
+        <f>$F68*IF($I68="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3694,6 +4542,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L69" s="4">
+        <f>$D69*IF($I69="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M69" s="4">
+        <f>$E69*IF($I69="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N69" s="4">
+        <f>$F69*IF($I69="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3741,6 +4601,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L70" s="4">
+        <f>$D70*IF($I70="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M70" s="4">
+        <f>$E70*IF($I70="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N70" s="4">
+        <f>$F70*IF($I70="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3788,6 +4660,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L71" s="4">
+        <f>$D71*IF($I71="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M71" s="4">
+        <f>$E71*IF($I71="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N71" s="4">
+        <f>$F71*IF($I71="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3835,6 +4719,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L72" s="4">
+        <f>$D72*IF($I72="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M72" s="4">
+        <f>$E72*IF($I72="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N72" s="4">
+        <f>$F72*IF($I72="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3882,6 +4778,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L73" s="4">
+        <f>$D73*IF($I73="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M73" s="4">
+        <f>$E73*IF($I73="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N73" s="4">
+        <f>$F73*IF($I73="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3929,6 +4837,18 @@
           <t>MT65</t>
         </is>
       </c>
+      <c r="L74" s="4">
+        <f>$D74*IF($I74="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M74" s="4">
+        <f>$E74*IF($I74="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N74" s="4">
+        <f>$F74*IF($I74="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3976,6 +4896,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L75" s="4">
+        <f>$D75*IF($I75="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M75" s="4">
+        <f>$E75*IF($I75="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N75" s="4">
+        <f>$F75*IF($I75="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4023,6 +4955,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L76" s="4">
+        <f>$D76*IF($I76="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M76" s="4">
+        <f>$E76*IF($I76="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N76" s="4">
+        <f>$F76*IF($I76="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4070,6 +5014,18 @@
           <t>NTE360</t>
         </is>
       </c>
+      <c r="L77" s="4">
+        <f>$D77*IF($I77="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M77" s="4">
+        <f>$E77*IF($I77="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N77" s="4">
+        <f>$F77*IF($I77="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4117,6 +5073,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L78" s="4">
+        <f>$D78*IF($I78="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M78" s="4">
+        <f>$E78*IF($I78="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N78" s="4">
+        <f>$F78*IF($I78="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4164,6 +5132,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L79" s="4">
+        <f>$D79*IF($I79="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M79" s="4">
+        <f>$E79*IF($I79="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N79" s="4">
+        <f>$F79*IF($I79="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4211,6 +5191,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L80" s="4">
+        <f>$D80*IF($I80="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M80" s="4">
+        <f>$E80*IF($I80="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N80" s="4">
+        <f>$F80*IF($I80="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4258,6 +5250,18 @@
           <t>930E-4SE</t>
         </is>
       </c>
+      <c r="L81" s="4">
+        <f>$D81*IF($I81="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M81" s="4">
+        <f>$E81*IF($I81="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N81" s="4">
+        <f>$F81*IF($I81="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4305,6 +5309,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L82" s="4">
+        <f>$D82*IF($I82="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M82" s="4">
+        <f>$E82*IF($I82="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N82" s="4">
+        <f>$F82*IF($I82="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4352,6 +5368,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L83" s="4">
+        <f>$D83*IF($I83="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M83" s="4">
+        <f>$E83*IF($I83="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N83" s="4">
+        <f>$F83*IF($I83="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4399,6 +5427,18 @@
           <t>EH4000AC-3</t>
         </is>
       </c>
+      <c r="L84" s="4">
+        <f>$D84*IF($I84="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M84" s="4">
+        <f>$E84*IF($I84="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N84" s="4">
+        <f>$F84*IF($I84="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4446,6 +5486,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L85" s="4">
+        <f>$D85*IF($I85="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M85" s="4">
+        <f>$E85*IF($I85="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N85" s="4">
+        <f>$F85*IF($I85="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4493,6 +5545,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L86" s="4">
+        <f>$D86*IF($I86="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M86" s="4">
+        <f>$E86*IF($I86="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N86" s="4">
+        <f>$F86*IF($I86="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4540,6 +5604,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L87" s="4">
+        <f>$D87*IF($I87="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M87" s="4">
+        <f>$E87*IF($I87="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N87" s="4">
+        <f>$F87*IF($I87="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4587,6 +5663,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L88" s="4">
+        <f>$D88*IF($I88="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M88" s="4">
+        <f>$E88*IF($I88="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N88" s="4">
+        <f>$F88*IF($I88="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4634,6 +5722,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L89" s="4">
+        <f>$D89*IF($I89="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M89" s="4">
+        <f>$E89*IF($I89="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N89" s="4">
+        <f>$F89*IF($I89="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4681,6 +5781,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L90" s="4">
+        <f>$D90*IF($I90="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M90" s="4">
+        <f>$E90*IF($I90="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N90" s="4">
+        <f>$F90*IF($I90="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4728,6 +5840,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L91" s="4">
+        <f>$D91*IF($I91="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M91" s="4">
+        <f>$E91*IF($I91="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N91" s="4">
+        <f>$F91*IF($I91="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4775,6 +5899,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L92" s="4">
+        <f>$D92*IF($I92="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M92" s="4">
+        <f>$E92*IF($I92="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N92" s="4">
+        <f>$F92*IF($I92="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4822,6 +5958,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L93" s="4">
+        <f>$D93*IF($I93="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M93" s="4">
+        <f>$E93*IF($I93="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N93" s="4">
+        <f>$F93*IF($I93="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4869,6 +6017,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L94" s="4">
+        <f>$D94*IF($I94="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M94" s="4">
+        <f>$E94*IF($I94="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N94" s="4">
+        <f>$F94*IF($I94="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4916,6 +6076,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L95" s="4">
+        <f>$D95*IF($I95="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M95" s="4">
+        <f>$E95*IF($I95="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N95" s="4">
+        <f>$F95*IF($I95="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4963,6 +6135,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L96" s="4">
+        <f>$D96*IF($I96="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M96" s="4">
+        <f>$E96*IF($I96="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N96" s="4">
+        <f>$F96*IF($I96="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5010,6 +6194,18 @@
           <t>793F</t>
         </is>
       </c>
+      <c r="L97" s="4">
+        <f>$D97*IF($I97="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M97" s="4">
+        <f>$E97*IF($I97="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N97" s="4">
+        <f>$F97*IF($I97="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5057,6 +6253,18 @@
           <t>793F</t>
         </is>
       </c>
+      <c r="L98" s="4">
+        <f>$D98*IF($I98="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M98" s="4">
+        <f>$E98*IF($I98="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N98" s="4">
+        <f>$F98*IF($I98="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5104,6 +6312,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L99" s="4">
+        <f>$D99*IF($I99="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M99" s="4">
+        <f>$E99*IF($I99="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N99" s="4">
+        <f>$F99*IF($I99="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5151,6 +6371,18 @@
           <t>793E</t>
         </is>
       </c>
+      <c r="L100" s="4">
+        <f>$D100*IF($I100="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M100" s="4">
+        <f>$E100*IF($I100="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N100" s="4">
+        <f>$F100*IF($I100="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5198,6 +6430,18 @@
           <t>795F</t>
         </is>
       </c>
+      <c r="L101" s="4">
+        <f>$D101*IF($I101="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M101" s="4">
+        <f>$E101*IF($I101="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N101" s="4">
+        <f>$F101*IF($I101="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5245,6 +6489,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L102" s="4">
+        <f>$D102*IF($I102="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M102" s="4">
+        <f>$E102*IF($I102="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N102" s="4">
+        <f>$F102*IF($I102="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5292,6 +6548,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L103" s="4">
+        <f>$D103*IF($I103="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M103" s="4">
+        <f>$E103*IF($I103="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N103" s="4">
+        <f>$F103*IF($I103="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5339,6 +6607,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L104" s="4">
+        <f>$D104*IF($I104="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M104" s="4">
+        <f>$E104*IF($I104="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N104" s="4">
+        <f>$F104*IF($I104="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5386,6 +6666,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L105" s="4">
+        <f>$D105*IF($I105="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M105" s="4">
+        <f>$E105*IF($I105="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N105" s="4">
+        <f>$F105*IF($I105="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5433,6 +6725,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L106" s="4">
+        <f>$D106*IF($I106="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M106" s="4">
+        <f>$E106*IF($I106="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N106" s="4">
+        <f>$F106*IF($I106="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5480,6 +6784,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L107" s="4">
+        <f>$D107*IF($I107="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M107" s="4">
+        <f>$E107*IF($I107="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N107" s="4">
+        <f>$F107*IF($I107="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5527,6 +6843,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L108" s="4">
+        <f>$D108*IF($I108="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M108" s="4">
+        <f>$E108*IF($I108="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N108" s="4">
+        <f>$F108*IF($I108="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5574,6 +6902,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L109" s="4">
+        <f>$D109*IF($I109="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M109" s="4">
+        <f>$E109*IF($I109="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N109" s="4">
+        <f>$F109*IF($I109="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5621,6 +6961,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L110" s="4">
+        <f>$D110*IF($I110="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M110" s="4">
+        <f>$E110*IF($I110="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N110" s="4">
+        <f>$F110*IF($I110="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5668,6 +7020,18 @@
           <t>830E-1AC</t>
         </is>
       </c>
+      <c r="L111" s="4">
+        <f>$D111*IF($I111="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M111" s="4">
+        <f>$E111*IF($I111="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N111" s="4">
+        <f>$F111*IF($I111="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5715,6 +7079,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L112" s="4">
+        <f>$D112*IF($I112="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M112" s="4">
+        <f>$E112*IF($I112="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N112" s="4">
+        <f>$F112*IF($I112="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5762,6 +7138,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L113" s="4">
+        <f>$D113*IF($I113="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M113" s="4">
+        <f>$E113*IF($I113="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N113" s="4">
+        <f>$F113*IF($I113="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5809,6 +7197,18 @@
           <t>830E-5</t>
         </is>
       </c>
+      <c r="L114" s="4">
+        <f>$D114*IF($I114="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M114" s="4">
+        <f>$E114*IF($I114="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N114" s="4">
+        <f>$F114*IF($I114="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5856,6 +7256,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L115" s="4">
+        <f>$D115*IF($I115="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M115" s="4">
+        <f>$E115*IF($I115="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N115" s="4">
+        <f>$F115*IF($I115="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5903,6 +7315,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L116" s="4">
+        <f>$D116*IF($I116="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M116" s="4">
+        <f>$E116*IF($I116="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N116" s="4">
+        <f>$F116*IF($I116="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5950,6 +7374,18 @@
           <t>930E-5</t>
         </is>
       </c>
+      <c r="L117" s="4">
+        <f>$D117*IF($I117="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M117" s="4">
+        <f>$E117*IF($I117="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N117" s="4">
+        <f>$F117*IF($I117="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5997,6 +7433,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L118" s="4">
+        <f>$D118*IF($I118="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M118" s="4">
+        <f>$E118*IF($I118="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N118" s="4">
+        <f>$F118*IF($I118="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6044,6 +7492,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L119" s="4">
+        <f>$D119*IF($I119="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M119" s="4">
+        <f>$E119*IF($I119="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N119" s="4">
+        <f>$F119*IF($I119="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6091,6 +7551,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L120" s="4">
+        <f>$D120*IF($I120="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M120" s="4">
+        <f>$E120*IF($I120="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N120" s="4">
+        <f>$F120*IF($I120="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6138,6 +7610,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L121" s="4">
+        <f>$D121*IF($I121="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M121" s="4">
+        <f>$E121*IF($I121="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N121" s="4">
+        <f>$F121*IF($I121="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6185,6 +7669,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L122" s="4">
+        <f>$D122*IF($I122="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M122" s="4">
+        <f>$E122*IF($I122="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N122" s="4">
+        <f>$F122*IF($I122="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6232,6 +7728,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L123" s="4">
+        <f>$D123*IF($I123="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M123" s="4">
+        <f>$E123*IF($I123="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N123" s="4">
+        <f>$F123*IF($I123="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6279,6 +7787,18 @@
           <t>830E</t>
         </is>
       </c>
+      <c r="L124" s="4">
+        <f>$D124*IF($I124="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M124" s="4">
+        <f>$E124*IF($I124="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N124" s="4">
+        <f>$F124*IF($I124="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6326,6 +7846,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L125" s="4">
+        <f>$D125*IF($I125="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M125" s="4">
+        <f>$E125*IF($I125="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N125" s="4">
+        <f>$F125*IF($I125="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6373,6 +7905,18 @@
           <t>TH663i</t>
         </is>
       </c>
+      <c r="L126" s="4">
+        <f>$D126*IF($I126="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M126" s="4">
+        <f>$E126*IF($I126="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N126" s="4">
+        <f>$F126*IF($I126="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6420,6 +7964,18 @@
           <t>930E</t>
         </is>
       </c>
+      <c r="L127" s="4">
+        <f>$D127*IF($I127="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M127" s="4">
+        <f>$E127*IF($I127="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N127" s="4">
+        <f>$F127*IF($I127="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6467,6 +8023,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L128" s="4">
+        <f>$D128*IF($I128="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M128" s="4">
+        <f>$E128*IF($I128="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N128" s="4">
+        <f>$F128*IF($I128="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6514,6 +8082,18 @@
           <t>777F</t>
         </is>
       </c>
+      <c r="L129" s="4">
+        <f>$D129*IF($I129="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M129" s="4">
+        <f>$E129*IF($I129="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N129" s="4">
+        <f>$F129*IF($I129="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6561,6 +8141,18 @@
           <t>789D</t>
         </is>
       </c>
+      <c r="L130" s="4">
+        <f>$D130*IF($I130="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M130" s="4">
+        <f>$E130*IF($I130="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N130" s="4">
+        <f>$F130*IF($I130="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6608,6 +8200,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L131" s="4">
+        <f>$D131*IF($I131="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M131" s="4">
+        <f>$E131*IF($I131="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N131" s="4">
+        <f>$F131*IF($I131="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6655,6 +8259,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L132" s="4">
+        <f>$D132*IF($I132="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M132" s="4">
+        <f>$E132*IF($I132="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N132" s="4">
+        <f>$F132*IF($I132="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6702,6 +8318,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L133" s="4">
+        <f>$D133*IF($I133="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M133" s="4">
+        <f>$E133*IF($I133="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N133" s="4">
+        <f>$F133*IF($I133="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6749,6 +8377,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L134" s="4">
+        <f>$D134*IF($I134="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M134" s="4">
+        <f>$E134*IF($I134="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N134" s="4">
+        <f>$F134*IF($I134="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6796,6 +8436,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L135" s="4">
+        <f>$D135*IF($I135="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M135" s="4">
+        <f>$E135*IF($I135="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N135" s="4">
+        <f>$F135*IF($I135="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6843,6 +8495,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L136" s="4">
+        <f>$D136*IF($I136="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M136" s="4">
+        <f>$E136*IF($I136="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N136" s="4">
+        <f>$F136*IF($I136="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6890,6 +8554,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L137" s="4">
+        <f>$D137*IF($I137="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M137" s="4">
+        <f>$E137*IF($I137="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N137" s="4">
+        <f>$F137*IF($I137="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6937,6 +8613,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L138" s="4">
+        <f>$D138*IF($I138="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M138" s="4">
+        <f>$E138*IF($I138="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N138" s="4">
+        <f>$F138*IF($I138="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6984,6 +8672,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L139" s="4">
+        <f>$D139*IF($I139="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M139" s="4">
+        <f>$E139*IF($I139="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N139" s="4">
+        <f>$F139*IF($I139="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7031,6 +8731,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L140" s="4">
+        <f>$D140*IF($I140="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M140" s="4">
+        <f>$E140*IF($I140="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N140" s="4">
+        <f>$F140*IF($I140="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7078,6 +8790,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L141" s="4">
+        <f>$D141*IF($I141="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M141" s="4">
+        <f>$E141*IF($I141="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N141" s="4">
+        <f>$F141*IF($I141="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7125,6 +8849,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L142" s="4">
+        <f>$D142*IF($I142="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M142" s="4">
+        <f>$E142*IF($I142="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N142" s="4">
+        <f>$F142*IF($I142="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7172,6 +8908,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L143" s="4">
+        <f>$D143*IF($I143="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M143" s="4">
+        <f>$E143*IF($I143="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N143" s="4">
+        <f>$F143*IF($I143="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7219,6 +8967,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L144" s="4">
+        <f>$D144*IF($I144="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M144" s="4">
+        <f>$E144*IF($I144="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N144" s="4">
+        <f>$F144*IF($I144="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7266,6 +9026,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L145" s="4">
+        <f>$D145*IF($I145="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M145" s="4">
+        <f>$E145*IF($I145="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N145" s="4">
+        <f>$F145*IF($I145="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7313,6 +9085,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L146" s="4">
+        <f>$D146*IF($I146="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M146" s="4">
+        <f>$E146*IF($I146="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N146" s="4">
+        <f>$F146*IF($I146="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7360,6 +9144,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L147" s="4">
+        <f>$D147*IF($I147="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M147" s="4">
+        <f>$E147*IF($I147="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N147" s="4">
+        <f>$F147*IF($I147="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7407,6 +9203,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L148" s="4">
+        <f>$D148*IF($I148="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M148" s="4">
+        <f>$E148*IF($I148="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N148" s="4">
+        <f>$F148*IF($I148="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7454,6 +9262,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L149" s="4">
+        <f>$D149*IF($I149="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M149" s="4">
+        <f>$E149*IF($I149="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N149" s="4">
+        <f>$F149*IF($I149="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7501,6 +9321,18 @@
           <t>785</t>
         </is>
       </c>
+      <c r="L150" s="4">
+        <f>$D150*IF($I150="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M150" s="4">
+        <f>$E150*IF($I150="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N150" s="4">
+        <f>$F150*IF($I150="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7548,6 +9380,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L151" s="4">
+        <f>$D151*IF($I151="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M151" s="4">
+        <f>$E151*IF($I151="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N151" s="4">
+        <f>$F151*IF($I151="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7595,6 +9439,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L152" s="4">
+        <f>$D152*IF($I152="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M152" s="4">
+        <f>$E152*IF($I152="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N152" s="4">
+        <f>$F152*IF($I152="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7642,6 +9498,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L153" s="4">
+        <f>$D153*IF($I153="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M153" s="4">
+        <f>$E153*IF($I153="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N153" s="4">
+        <f>$F153*IF($I153="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7689,6 +9557,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L154" s="4">
+        <f>$D154*IF($I154="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M154" s="4">
+        <f>$E154*IF($I154="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N154" s="4">
+        <f>$F154*IF($I154="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7736,6 +9616,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L155" s="4">
+        <f>$D155*IF($I155="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M155" s="4">
+        <f>$E155*IF($I155="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N155" s="4">
+        <f>$F155*IF($I155="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7783,6 +9675,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L156" s="4">
+        <f>$D156*IF($I156="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M156" s="4">
+        <f>$E156*IF($I156="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N156" s="4">
+        <f>$F156*IF($I156="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7830,6 +9734,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L157" s="4">
+        <f>$D157*IF($I157="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M157" s="4">
+        <f>$E157*IF($I157="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N157" s="4">
+        <f>$F157*IF($I157="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7877,6 +9793,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L158" s="4">
+        <f>$D158*IF($I158="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M158" s="4">
+        <f>$E158*IF($I158="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N158" s="4">
+        <f>$F158*IF($I158="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7924,6 +9852,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L159" s="4">
+        <f>$D159*IF($I159="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M159" s="4">
+        <f>$E159*IF($I159="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N159" s="4">
+        <f>$F159*IF($I159="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7971,6 +9911,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L160" s="4">
+        <f>$D160*IF($I160="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M160" s="4">
+        <f>$E160*IF($I160="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N160" s="4">
+        <f>$F160*IF($I160="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8018,6 +9970,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L161" s="4">
+        <f>$D161*IF($I161="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M161" s="4">
+        <f>$E161*IF($I161="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N161" s="4">
+        <f>$F161*IF($I161="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8065,6 +10029,18 @@
           <t>785D</t>
         </is>
       </c>
+      <c r="L162" s="4">
+        <f>$D162*IF($I162="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M162" s="4">
+        <f>$E162*IF($I162="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N162" s="4">
+        <f>$F162*IF($I162="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8112,6 +10088,18 @@
           <t>777E</t>
         </is>
       </c>
+      <c r="L163" s="4">
+        <f>$D163*IF($I163="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M163" s="4">
+        <f>$E163*IF($I163="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N163" s="4">
+        <f>$F163*IF($I163="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8159,6 +10147,18 @@
           <t>777E</t>
         </is>
       </c>
+      <c r="L164" s="4">
+        <f>$D164*IF($I164="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M164" s="4">
+        <f>$E164*IF($I164="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N164" s="4">
+        <f>$F164*IF($I164="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8206,6 +10206,18 @@
           <t>777E</t>
         </is>
       </c>
+      <c r="L165" s="4">
+        <f>$D165*IF($I165="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M165" s="4">
+        <f>$E165*IF($I165="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N165" s="4">
+        <f>$F165*IF($I165="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8253,6 +10265,18 @@
           <t>777E</t>
         </is>
       </c>
+      <c r="L166" s="4">
+        <f>$D166*IF($I166="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M166" s="4">
+        <f>$E166*IF($I166="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N166" s="4">
+        <f>$F166*IF($I166="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8300,6 +10324,18 @@
           <t>777</t>
         </is>
       </c>
+      <c r="L167" s="4">
+        <f>$D167*IF($I167="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M167" s="4">
+        <f>$E167*IF($I167="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N167" s="4">
+        <f>$F167*IF($I167="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8347,6 +10383,18 @@
           <t>777E</t>
         </is>
       </c>
+      <c r="L168" s="4">
+        <f>$D168*IF($I168="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M168" s="4">
+        <f>$E168*IF($I168="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N168" s="4">
+        <f>$F168*IF($I168="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8394,6 +10442,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L169" s="4">
+        <f>$D169*IF($I169="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M169" s="4">
+        <f>$E169*IF($I169="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N169" s="4">
+        <f>$F169*IF($I169="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8441,6 +10501,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L170" s="4">
+        <f>$D170*IF($I170="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M170" s="4">
+        <f>$E170*IF($I170="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N170" s="4">
+        <f>$F170*IF($I170="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8488,6 +10560,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L171" s="4">
+        <f>$D171*IF($I171="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M171" s="4">
+        <f>$E171*IF($I171="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N171" s="4">
+        <f>$F171*IF($I171="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8535,6 +10619,18 @@
           <t>EH4000AC-3</t>
         </is>
       </c>
+      <c r="L172" s="4">
+        <f>$D172*IF($I172="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M172" s="4">
+        <f>$E172*IF($I172="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N172" s="4">
+        <f>$F172*IF($I172="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8582,6 +10678,18 @@
           <t>785C</t>
         </is>
       </c>
+      <c r="L173" s="4">
+        <f>$D173*IF($I173="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M173" s="4">
+        <f>$E173*IF($I173="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N173" s="4">
+        <f>$F173*IF($I173="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8629,6 +10737,18 @@
           <t>785C</t>
         </is>
       </c>
+      <c r="L174" s="4">
+        <f>$D174*IF($I174="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M174" s="4">
+        <f>$E174*IF($I174="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N174" s="4">
+        <f>$F174*IF($I174="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8676,6 +10796,18 @@
           <t>EH4000AC-3</t>
         </is>
       </c>
+      <c r="L175" s="4">
+        <f>$D175*IF($I175="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M175" s="4">
+        <f>$E175*IF($I175="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N175" s="4">
+        <f>$F175*IF($I175="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8723,6 +10855,18 @@
           <t>785C</t>
         </is>
       </c>
+      <c r="L176" s="4">
+        <f>$D176*IF($I176="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M176" s="4">
+        <f>$E176*IF($I176="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N176" s="4">
+        <f>$F176*IF($I176="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8770,6 +10914,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L177" s="4">
+        <f>$D177*IF($I177="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M177" s="4">
+        <f>$E177*IF($I177="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N177" s="4">
+        <f>$F177*IF($I177="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8817,6 +10973,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L178" s="4">
+        <f>$D178*IF($I178="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M178" s="4">
+        <f>$E178*IF($I178="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N178" s="4">
+        <f>$F178*IF($I178="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8864,6 +11032,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L179" s="4">
+        <f>$D179*IF($I179="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M179" s="4">
+        <f>$E179*IF($I179="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N179" s="4">
+        <f>$F179*IF($I179="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8911,6 +11091,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L180" s="4">
+        <f>$D180*IF($I180="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M180" s="4">
+        <f>$E180*IF($I180="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N180" s="4">
+        <f>$F180*IF($I180="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -8958,6 +11150,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L181" s="4">
+        <f>$D181*IF($I181="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M181" s="4">
+        <f>$E181*IF($I181="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N181" s="4">
+        <f>$F181*IF($I181="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -9005,6 +11209,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L182" s="4">
+        <f>$D182*IF($I182="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M182" s="4">
+        <f>$E182*IF($I182="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N182" s="4">
+        <f>$F182*IF($I182="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9052,6 +11268,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L183" s="4">
+        <f>$D183*IF($I183="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M183" s="4">
+        <f>$E183*IF($I183="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N183" s="4">
+        <f>$F183*IF($I183="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -9099,6 +11327,18 @@
           <t>HD785-7</t>
         </is>
       </c>
+      <c r="L184" s="4">
+        <f>$D184*IF($I184="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M184" s="4">
+        <f>$E184*IF($I184="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N184" s="4">
+        <f>$F184*IF($I184="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9146,9 +11386,102 @@
           <t>930E-4</t>
         </is>
       </c>
+      <c r="L185" s="4">
+        <f>$D185*IF($I185="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="M185" s="4">
+        <f>$E185*IF($I185="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
+      <c r="N185" s="4">
+        <f>$F185*IF($I185="AUD",Assumptions!$B$2,Assumptions!$B$3)*Assumptions!$B$4</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K185"/>
+  <autoFilter ref="A1:N185"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>AUD to USD rate</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Applied to AUD rows. Edit B2 to refresh every sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>USD to USD</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>No conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>USD to IDR rate</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>17500</v>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Applied to all USD Value to get Value IDR. Edit B4 to refresh every sheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify Komatsu and Caterpillar model names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ReNvkBKePFXKJiXPJLaYQp
</commit_message>
<xml_diff>
--- a/PPT_Freight_Insurance_FOB.xlsx
+++ b/PPT_Freight_Insurance_FOB.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L2" s="4">
@@ -645,7 +645,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L3" s="4">
@@ -704,7 +704,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L4" s="4">
@@ -763,7 +763,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L5" s="4">
@@ -822,7 +822,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L6" s="4">
@@ -881,7 +881,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L7" s="4">
@@ -940,7 +940,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L8" s="4">
@@ -999,7 +999,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L9" s="4">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L10" s="4">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L11" s="4">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L12" s="4">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L13" s="4">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L14" s="4">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L15" s="4">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L16" s="4">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L17" s="4">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L18" s="4">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L19" s="4">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L20" s="4">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L21" s="4">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L22" s="4">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>930E-5</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L23" s="4">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L24" s="4">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>930E-5</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L25" s="4">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L26" s="4">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L28" s="4">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L29" s="4">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L30" s="4">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>777G</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L31" s="4">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L32" s="4">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L33" s="4">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L34" s="4">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L35" s="4">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L36" s="4">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L37" s="4">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L38" s="4">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L39" s="4">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L40" s="4">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L41" s="4">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>930E-5</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L42" s="4">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>930E-5</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L43" s="4">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L44" s="4">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>930E-5</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L45" s="4">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L46" s="4">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L47" s="4">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L48" s="4">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L49" s="4">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L50" s="4">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L51" s="4">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L52" s="4">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L53" s="4">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L56" s="4">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L66" s="4">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L67" s="4">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L73" s="4">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L78" s="4">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>930E-4SE</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L81" s="4">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L85" s="4">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L86" s="4">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L88" s="4">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L90" s="4">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>793F</t>
+          <t>793</t>
         </is>
       </c>
       <c r="L97" s="4">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>793F</t>
+          <t>793</t>
         </is>
       </c>
       <c r="L98" s="4">
@@ -6368,7 +6368,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>793E</t>
+          <t>793</t>
         </is>
       </c>
       <c r="L100" s="4">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>795F</t>
+          <t>795</t>
         </is>
       </c>
       <c r="L101" s="4">
@@ -6781,7 +6781,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L107" s="4">
@@ -7017,7 +7017,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>830E-1AC</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L111" s="4">
@@ -7076,7 +7076,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L112" s="4">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>830E-5</t>
+          <t>830E</t>
         </is>
       </c>
       <c r="L114" s="4">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>930E-5</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L117" s="4">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L128" s="4">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>777F</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L129" s="4">
@@ -8138,7 +8138,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>789D</t>
+          <t>789</t>
         </is>
       </c>
       <c r="L130" s="4">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L131" s="4">
@@ -8728,7 +8728,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L140" s="4">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L141" s="4">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L142" s="4">
@@ -8905,7 +8905,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L143" s="4">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L144" s="4">
@@ -9023,7 +9023,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L145" s="4">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L146" s="4">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L147" s="4">
@@ -9200,7 +9200,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L148" s="4">
@@ -9377,7 +9377,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L151" s="4">
@@ -9436,7 +9436,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L152" s="4">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L153" s="4">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L154" s="4">
@@ -9613,7 +9613,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L155" s="4">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L156" s="4">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L157" s="4">
@@ -9790,7 +9790,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L158" s="4">
@@ -9849,7 +9849,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L159" s="4">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L160" s="4">
@@ -9967,7 +9967,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L161" s="4">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>785D</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L162" s="4">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>777E</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L163" s="4">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>777E</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L164" s="4">
@@ -10203,7 +10203,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>777E</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L165" s="4">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>777E</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L166" s="4">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>777E</t>
+          <t>777</t>
         </is>
       </c>
       <c r="L168" s="4">
@@ -10439,7 +10439,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L169" s="4">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L170" s="4">
@@ -10557,7 +10557,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L171" s="4">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L173" s="4">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L174" s="4">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>785C</t>
+          <t>785</t>
         </is>
       </c>
       <c r="L176" s="4">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L177" s="4">
@@ -10970,7 +10970,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L178" s="4">
@@ -11029,7 +11029,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L179" s="4">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L180" s="4">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L181" s="4">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L182" s="4">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L183" s="4">
@@ -11324,7 +11324,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>HD785-7</t>
+          <t>HD785</t>
         </is>
       </c>
       <c r="L184" s="4">
@@ -11383,7 +11383,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>930E-4</t>
+          <t>930E</t>
         </is>
       </c>
       <c r="L185" s="4">

</xml_diff>

<commit_message>
Restore HD785-7 model name
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ReNvkBKePFXKJiXPJLaYQp
</commit_message>
<xml_diff>
--- a/PPT_Freight_Insurance_FOB.xlsx
+++ b/PPT_Freight_Insurance_FOB.xlsx
@@ -8020,7 +8020,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L128" s="4">
@@ -8728,7 +8728,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L140" s="4">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L141" s="4">
@@ -8846,7 +8846,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L142" s="4">
@@ -8905,7 +8905,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L143" s="4">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L144" s="4">
@@ -9023,7 +9023,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L145" s="4">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L146" s="4">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L147" s="4">
@@ -9200,7 +9200,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L148" s="4">
@@ -10439,7 +10439,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L169" s="4">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L170" s="4">
@@ -10557,7 +10557,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L171" s="4">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L177" s="4">
@@ -10970,7 +10970,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L178" s="4">
@@ -11029,7 +11029,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L179" s="4">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L180" s="4">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L181" s="4">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L182" s="4">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L183" s="4">
@@ -11324,7 +11324,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>HD785</t>
+          <t>HD785-7</t>
         </is>
       </c>
       <c r="L184" s="4">

</xml_diff>